<commit_message>
Stage 8 review fixes: HO-009
</commit_message>
<xml_diff>
--- a/output/archive/Tarnovell_Group/Brand/Migration/2026/Brand_Migration_Status_2026-09.xlsx
+++ b/output/archive/Tarnovell_Group/Brand/Migration/2026/Brand_Migration_Status_2026-09.xlsx
@@ -148,7 +148,7 @@
   <commentList>
     <comment ref="D14" authorId="0" shapeId="0">
       <text>
-        <t>Legacy Osterquill client and study documents are not to be restyled. Only the group-facing materials are in scope for G after completion.</t>
+        <t>Osterquill has not joined as at this snapshot. After completion, legacy client and study documents remain as issued; group-facing materials require approved brand and access decisions.</t>
       </text>
     </comment>
   </commentList>
@@ -482,7 +482,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Tarnovell Brand Guidelines v1 (February 2020), as updated for the common master</t>
+          <t>HO-015: Tarnovell Brand Guidelines v1 (February 2020); archive reference: Tarnovell_Group/Brand/Guidelines/2020/Tarnovell_Brand_Guidelines_v1.docx. Use the controlled approved master for current subsidiary lines.</t>
         </is>
       </c>
     </row>
@@ -519,12 +519,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Brand adoption</t>
+          <t>Common-master adoption</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Materials on common master</t>
+          <t>Master available</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Formulation SOP headers, two sets of slide decks, website footer</t>
+          <t>Formulation SOP headers, slide decks, website footer</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Legacy</t>
+          <t>Pre-completion / legacy</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Held apart. No changes until the archive is mapped and access is agreed</t>
+          <t>Not yet a group firm. Completion scheduled 01/10/2026; subsequent onboarding awaits access and QA mapping.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Update slide masters for the two Durnesswick decks</t>
+          <t>Update slide masters for remaining Durnesswick decks</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Two signatures still carry the earlier firm line</t>
+          <t>Confirm remaining signatures against the approved subsidiary line.</t>
         </is>
       </c>
     </row>

</xml_diff>